<commit_message>
chore(dados): regenera dossies e auditorias de completude dos 69 devedores
Dossies multiformato (html/json/md/xlsx) e AUDITORIA_* regenerados em sessoes anteriores; consultas.py ajustado; gerar_painel_web.py novo; .mcp.json registra servidor semgrep (sem segredos).
</commit_message>
<xml_diff>
--- a/DOSSIES_MULTIFORMATO/FENIXSOFT/dossie.xlsx
+++ b/DOSSIES_MULTIFORMATO/FENIXSOFT/dossie.xlsx
@@ -535,7 +535,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -547,7 +547,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -583,7 +583,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2029-10-01</t>
+          <t>2027-02-28</t>
         </is>
       </c>
     </row>

</xml_diff>